<commit_message>
cambio de seman fecha
</commit_message>
<xml_diff>
--- a/data/objetivos.xlsx
+++ b/data/objetivos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mariposacbc-my.sharepoint.com/personal/controladormultiemp_grupoclc_com/Documents/Documents/GitHub/JESKELL-TV/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="159" documentId="8_{4DF11E83-7A7F-4557-9B8C-6F15B10F53BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5492636A-E22D-4073-A4F4-05B8140EA168}"/>
+  <xr:revisionPtr revIDLastSave="160" documentId="8_{4DF11E83-7A7F-4557-9B8C-6F15B10F53BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2602FDEA-5147-414D-9057-3F6DE7C10C98}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -225,7 +225,7 @@
     <t>En ejecucion</t>
   </si>
   <si>
-    <t>14/09/2026 al 20/09/2026</t>
+    <t>21/09/2026 al 27/09/2026</t>
   </si>
 </sst>
 </file>
@@ -539,7 +539,7 @@
     <xf numFmtId="17" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -547,10 +547,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -869,14 +869,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="28"/>
       <c r="C1" s="28"/>
     </row>
     <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="31"/>
+      <c r="A2" s="32"/>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
     </row>
@@ -1106,23 +1106,23 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="27"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="28"/>
       <c r="C27" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A18:C18"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A18:C18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1141,7 +1141,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="27" t="s">
         <v>40</v>
       </c>
       <c r="B1" s="28"/>
@@ -1150,7 +1150,7 @@
       <c r="E1" s="28"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="31"/>
+      <c r="A2" s="32"/>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
       <c r="D2" s="28"/>

</xml_diff>

<commit_message>
actualizacion de meta semanal
</commit_message>
<xml_diff>
--- a/data/objetivos.xlsx
+++ b/data/objetivos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mariposacbc-my.sharepoint.com/personal/controladormultiemp_grupoclc_com/Documents/Documents/GitHub/JESKELL-TV/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="180" documentId="8_{4DF11E83-7A7F-4557-9B8C-6F15B10F53BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4D9A08A-9E6D-4A1D-B61F-EE95B050772F}"/>
+  <xr:revisionPtr revIDLastSave="197" documentId="8_{4DF11E83-7A7F-4557-9B8C-6F15B10F53BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87C47C7C-F00F-4CE8-B613-E5B41F3A31B5}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="SEMANA" sheetId="1" r:id="rId1"/>
     <sheet name="PRODUCCION_MENSUAL" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -216,10 +216,10 @@
     <t>Excelente Semana</t>
   </si>
   <si>
-    <t>28/09/2026 al 4/10/2026</t>
-  </si>
-  <si>
     <t>Octubre</t>
+  </si>
+  <si>
+    <t>5/10/2026 al 11/10/2026</t>
   </si>
 </sst>
 </file>
@@ -457,7 +457,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -533,22 +533,25 @@
     <xf numFmtId="17" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -863,14 +866,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="28"/>
       <c r="C1" s="28"/>
     </row>
     <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="27"/>
+      <c r="A2" s="32"/>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
     </row>
@@ -890,7 +893,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>5</v>
@@ -901,7 +904,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>7</v>
@@ -919,18 +922,18 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
     </row>
     <row r="8" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B8" s="3">
-        <v>28320</v>
+        <v>62960</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>12</v>
@@ -941,18 +944,18 @@
         <v>13</v>
       </c>
       <c r="B9" s="3">
-        <v>28320</v>
+        <v>79968</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
     </row>
     <row r="11" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
@@ -966,11 +969,11 @@
       </c>
     </row>
     <row r="12" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
     </row>
     <row r="13" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
@@ -984,11 +987,11 @@
       </c>
     </row>
     <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="32"/>
-      <c r="C14" s="32"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
     </row>
     <row r="15" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
@@ -1002,11 +1005,11 @@
       </c>
     </row>
     <row r="16" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
     </row>
     <row r="17" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
@@ -1020,11 +1023,11 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
     </row>
     <row r="19" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
@@ -1063,11 +1066,11 @@
       </c>
     </row>
     <row r="22" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="31" t="s">
+      <c r="A22" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="32"/>
-      <c r="C22" s="32"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
     </row>
     <row r="23" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
@@ -1081,11 +1084,11 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="31" t="s">
+      <c r="A24" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="32"/>
-      <c r="C24" s="32"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
     </row>
     <row r="25" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
@@ -1099,7 +1102,7 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="33"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="28"/>
       <c r="C27" s="28"/>
     </row>
@@ -1134,7 +1137,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>40</v>
       </c>
       <c r="B1" s="28"/>
@@ -1143,7 +1146,7 @@
       <c r="E1" s="28"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="27"/>
+      <c r="A2" s="32"/>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
       <c r="D2" s="28"/>
@@ -1284,7 +1287,7 @@
       <c r="C12" s="19">
         <v>205178</v>
       </c>
-      <c r="D12" s="15"/>
+      <c r="D12" s="34"/>
       <c r="E12" s="22"/>
     </row>
     <row r="13" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -1295,7 +1298,7 @@
         <v>359998</v>
       </c>
       <c r="C13" s="19">
-        <v>28320</v>
+        <v>79968</v>
       </c>
       <c r="D13" s="15"/>
       <c r="E13" s="16"/>
@@ -1319,7 +1322,7 @@
       <c r="E15" s="16"/>
     </row>
     <row r="17" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="30"/>
+      <c r="A17" s="33"/>
       <c r="B17" s="28"/>
       <c r="C17" s="28"/>
       <c r="D17" s="28"/>

</xml_diff>